<commit_message>
dados: 2026-10-23 08:25 (132 arquivos)
</commit_message>
<xml_diff>
--- a/xlsx/contratos/latest.xlsx
+++ b/xlsx/contratos/latest.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4046" uniqueCount="1405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4046" uniqueCount="1406">
   <si>
     <t>Contrato</t>
   </si>
@@ -2967,73 +2967,76 @@
     <t>16/10/2026</t>
   </si>
   <si>
+    <t>1051 - Claudio Wasserman - 17/10/26</t>
+  </si>
+  <si>
+    <t>Claudio Wasserman</t>
+  </si>
+  <si>
+    <t>R$ 50900.00</t>
+  </si>
+  <si>
+    <t>17/12/2026</t>
+  </si>
+  <si>
+    <t>1044 - MO REGINA RURIKO - 14/10/26</t>
+  </si>
+  <si>
+    <t>REGINA RURIKO TATEIGI</t>
+  </si>
+  <si>
+    <t>R$ 29700.00</t>
+  </si>
+  <si>
+    <t>19/10/2026</t>
+  </si>
+  <si>
+    <t>1023 - Thiago Degola - 25/09/26</t>
+  </si>
+  <si>
+    <t>Thiago Souza Dias Degola</t>
+  </si>
+  <si>
+    <t>1029 - CARLA EMÍLIA DE OLIVEIRA SOUZA FERREIRA - 01/10/26</t>
+  </si>
+  <si>
+    <t>CARLA EMÍLIA DE OLIVEIRA SOUZA FERREIRA</t>
+  </si>
+  <si>
+    <t>R$ 178.08</t>
+  </si>
+  <si>
+    <t>07/10/2026</t>
+  </si>
+  <si>
+    <t>15/12/2026</t>
+  </si>
+  <si>
+    <t>1009 - Mariana Andrade Derossi - 17/09/26</t>
+  </si>
+  <si>
+    <t>Mariana Andrade Derossi</t>
+  </si>
+  <si>
+    <t>R$ 67698.84</t>
+  </si>
+  <si>
+    <t>18/02/2027</t>
+  </si>
+  <si>
+    <t>1048 - Venda Avulsa - VIVIAN MOURA BENIFICA GAZOLA</t>
+  </si>
+  <si>
+    <t>VIVIAN MOURA BENIFICA GAZOLA</t>
+  </si>
+  <si>
+    <t>R$ 340.52</t>
+  </si>
+  <si>
+    <t>15/10/2026</t>
+  </si>
+  <si>
     <t>23/12/2026</t>
-  </si>
-  <si>
-    <t>1051 - Claudio Wasserman - 17/10/26</t>
-  </si>
-  <si>
-    <t>Claudio Wasserman</t>
-  </si>
-  <si>
-    <t>R$ 50900.00</t>
-  </si>
-  <si>
-    <t>1044 - MO REGINA RURIKO - 14/10/26</t>
-  </si>
-  <si>
-    <t>REGINA RURIKO TATEIGI</t>
-  </si>
-  <si>
-    <t>R$ 29700.00</t>
-  </si>
-  <si>
-    <t>19/10/2026</t>
-  </si>
-  <si>
-    <t>1023 - Thiago Degola - 25/09/26</t>
-  </si>
-  <si>
-    <t>Thiago Souza Dias Degola</t>
-  </si>
-  <si>
-    <t>1029 - CARLA EMÍLIA DE OLIVEIRA SOUZA FERREIRA - 01/10/26</t>
-  </si>
-  <si>
-    <t>CARLA EMÍLIA DE OLIVEIRA SOUZA FERREIRA</t>
-  </si>
-  <si>
-    <t>R$ 178.08</t>
-  </si>
-  <si>
-    <t>07/10/2026</t>
-  </si>
-  <si>
-    <t>15/12/2026</t>
-  </si>
-  <si>
-    <t>1009 - Mariana Andrade Derossi - 17/09/26</t>
-  </si>
-  <si>
-    <t>Mariana Andrade Derossi</t>
-  </si>
-  <si>
-    <t>R$ 67698.84</t>
-  </si>
-  <si>
-    <t>18/02/2027</t>
-  </si>
-  <si>
-    <t>1048 - Venda Avulsa - VIVIAN MOURA BENIFICA GAZOLA</t>
-  </si>
-  <si>
-    <t>VIVIAN MOURA BENIFICA GAZOLA</t>
-  </si>
-  <si>
-    <t>R$ 340.52</t>
-  </si>
-  <si>
-    <t>15/10/2026</t>
   </si>
   <si>
     <t>1047 - Patrícia Santos da Silva - 15/10/26</t>
@@ -13717,7 +13720,7 @@
         <v>983</v>
       </c>
       <c r="J288" t="s">
-        <v>984</v>
+        <v>957</v>
       </c>
       <c r="K288" t="s">
         <v>2</v>
@@ -13763,10 +13766,10 @@
         <v>105101.0</v>
       </c>
       <c r="B290" t="s">
+        <v>984</v>
+      </c>
+      <c r="C290" t="s">
         <v>985</v>
-      </c>
-      <c r="C290" t="s">
-        <v>986</v>
       </c>
       <c r="D290" t="s">
         <v>69</v>
@@ -13778,7 +13781,7 @@
         <v>52</v>
       </c>
       <c r="G290" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="H290" t="s">
         <v>38</v>
@@ -13787,7 +13790,7 @@
         <v>915</v>
       </c>
       <c r="J290" t="s">
-        <v>98</v>
+        <v>987</v>
       </c>
       <c r="K290" t="s">
         <v>2</v>
@@ -13962,7 +13965,7 @@
         <v>1006</v>
       </c>
       <c r="J295" t="s">
-        <v>984</v>
+        <v>1007</v>
       </c>
       <c r="K295" t="s">
         <v>2</v>
@@ -13973,7 +13976,7 @@
         <v>104701.0</v>
       </c>
       <c r="B296" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="C296" t="s">
         <v>795</v>
@@ -13988,7 +13991,7 @@
         <v>45</v>
       </c>
       <c r="G296" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="H296" t="s">
         <v>38</v>
@@ -13997,7 +14000,7 @@
         <v>1006</v>
       </c>
       <c r="J296" t="s">
-        <v>984</v>
+        <v>1007</v>
       </c>
       <c r="K296" t="s">
         <v>2</v>
@@ -14008,7 +14011,7 @@
         <v>103501.0</v>
       </c>
       <c r="B297" t="s">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="C297" t="s">
         <v>597</v>
@@ -14023,7 +14026,7 @@
         <v>45</v>
       </c>
       <c r="G297" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="H297" t="s">
         <v>38</v>
@@ -14043,10 +14046,10 @@
         <v>103801.0</v>
       </c>
       <c r="B298" t="s">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="C298" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="D298" t="s">
         <v>146</v>
@@ -14058,7 +14061,7 @@
         <v>45</v>
       </c>
       <c r="G298" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="H298" t="s">
         <v>38</v>
@@ -14067,7 +14070,7 @@
         <v>1006</v>
       </c>
       <c r="J298" t="s">
-        <v>984</v>
+        <v>1007</v>
       </c>
       <c r="K298" t="s">
         <v>2</v>
@@ -14078,10 +14081,10 @@
         <v>92901.0</v>
       </c>
       <c r="B299" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="C299" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="D299" t="s">
         <v>69</v>
@@ -14093,7 +14096,7 @@
         <v>45</v>
       </c>
       <c r="G299" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="H299" t="s">
         <v>38</v>
@@ -14113,10 +14116,10 @@
         <v>95301.0</v>
       </c>
       <c r="B300" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="C300" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="D300" t="s">
         <v>159</v>
@@ -14128,16 +14131,16 @@
         <v>45</v>
       </c>
       <c r="G300" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="H300" t="s">
         <v>38</v>
       </c>
       <c r="I300" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
       <c r="J300" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
       <c r="K300" t="s">
         <v>2</v>
@@ -14148,10 +14151,10 @@
         <v>95001.0</v>
       </c>
       <c r="B301" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="C301" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
       <c r="D301" t="s">
         <v>43</v>
@@ -14169,7 +14172,7 @@
         <v>47</v>
       </c>
       <c r="I301" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="J301" t="s">
         <v>49</v>
@@ -14183,10 +14186,10 @@
         <v>94401.0</v>
       </c>
       <c r="B302" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
       <c r="C302" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="D302" t="s">
         <v>69</v>
@@ -14204,7 +14207,7 @@
         <v>38</v>
       </c>
       <c r="I302" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="J302" t="s">
         <v>957</v>
@@ -14218,7 +14221,7 @@
         <v>96401.0</v>
       </c>
       <c r="B303" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="C303" t="s">
         <v>765</v>
@@ -14233,16 +14236,16 @@
         <v>45</v>
       </c>
       <c r="G303" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="H303" t="s">
         <v>38</v>
       </c>
       <c r="I303" t="s">
-        <v>1030</v>
+        <v>1031</v>
       </c>
       <c r="J303" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="K303" t="s">
         <v>2</v>
@@ -14253,7 +14256,7 @@
         <v>96801.0</v>
       </c>
       <c r="B304" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="C304" t="s">
         <v>96</v>
@@ -14268,16 +14271,16 @@
         <v>45</v>
       </c>
       <c r="G304" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="H304" t="s">
         <v>38</v>
       </c>
       <c r="I304" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="J304" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="K304" t="s">
         <v>2</v>
@@ -14288,7 +14291,7 @@
         <v>97301.0</v>
       </c>
       <c r="B305" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="C305" t="s">
         <v>838</v>
@@ -14303,7 +14306,7 @@
         <v>45</v>
       </c>
       <c r="G305" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
       <c r="H305" t="s">
         <v>38</v>
@@ -14312,7 +14315,7 @@
         <v>859</v>
       </c>
       <c r="J305" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="K305" t="s">
         <v>2</v>
@@ -14323,7 +14326,7 @@
         <v>94301.0</v>
       </c>
       <c r="B306" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="C306" t="s">
         <v>861</v>
@@ -14344,10 +14347,10 @@
         <v>38</v>
       </c>
       <c r="I306" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="J306" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="K306" t="s">
         <v>2</v>
@@ -14358,10 +14361,10 @@
         <v>93701.0</v>
       </c>
       <c r="B307" t="s">
-        <v>1042</v>
+        <v>1043</v>
       </c>
       <c r="C307" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="D307" t="s">
         <v>69</v>
@@ -14373,7 +14376,7 @@
         <v>45</v>
       </c>
       <c r="G307" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="H307" t="s">
         <v>38</v>
@@ -14393,10 +14396,10 @@
         <v>91901.0</v>
       </c>
       <c r="B308" t="s">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="C308" t="s">
-        <v>1044</v>
+        <v>1045</v>
       </c>
       <c r="D308" t="s">
         <v>69</v>
@@ -14408,7 +14411,7 @@
         <v>52</v>
       </c>
       <c r="G308" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
       <c r="H308" t="s">
         <v>47</v>
@@ -14428,10 +14431,10 @@
         <v>92301.0</v>
       </c>
       <c r="B309" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="C309" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="D309" t="s">
         <v>69</v>
@@ -14449,7 +14452,7 @@
         <v>38</v>
       </c>
       <c r="I309" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="J309" t="s">
         <v>586</v>
@@ -14463,7 +14466,7 @@
         <v>93401.0</v>
       </c>
       <c r="B310" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="C310" t="s">
         <v>869</v>
@@ -14478,16 +14481,16 @@
         <v>45</v>
       </c>
       <c r="G310" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="H310" t="s">
         <v>38</v>
       </c>
       <c r="I310" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="J310" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="K310" t="s">
         <v>2</v>
@@ -14533,7 +14536,7 @@
         <v>95701.0</v>
       </c>
       <c r="B312" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="C312" t="s">
         <v>191</v>
@@ -14548,16 +14551,16 @@
         <v>45</v>
       </c>
       <c r="G312" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="H312" t="s">
         <v>38</v>
       </c>
       <c r="I312" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
       <c r="J312" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="K312" t="s">
         <v>2</v>
@@ -14568,10 +14571,10 @@
         <v>98701.0</v>
       </c>
       <c r="B313" t="s">
-        <v>1054</v>
+        <v>1055</v>
       </c>
       <c r="C313" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
       <c r="D313" t="s">
         <v>839</v>
@@ -14589,7 +14592,7 @@
         <v>38</v>
       </c>
       <c r="I313" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
       <c r="J313" t="s">
         <v>788</v>
@@ -14603,7 +14606,7 @@
         <v>99401.0</v>
       </c>
       <c r="B314" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="C314" t="s">
         <v>829</v>
@@ -14624,10 +14627,10 @@
         <v>38</v>
       </c>
       <c r="I314" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
       <c r="J314" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
       <c r="K314" t="s">
         <v>2</v>
@@ -14638,10 +14641,10 @@
         <v>95401.0</v>
       </c>
       <c r="B315" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="C315" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
       <c r="D315" t="s">
         <v>839</v>
@@ -14653,13 +14656,13 @@
         <v>45</v>
       </c>
       <c r="G315" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H315" t="s">
         <v>38</v>
       </c>
       <c r="I315" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
       <c r="J315" t="s">
         <v>586</v>
@@ -14673,7 +14676,7 @@
         <v>96901.0</v>
       </c>
       <c r="B316" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="C316" t="s">
         <v>305</v>
@@ -14688,13 +14691,13 @@
         <v>45</v>
       </c>
       <c r="G316" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="H316" t="s">
         <v>38</v>
       </c>
       <c r="I316" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="J316" t="s">
         <v>586</v>
@@ -14708,10 +14711,10 @@
         <v>96101.0</v>
       </c>
       <c r="B317" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="C317" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="D317" t="s">
         <v>839</v>
@@ -14723,7 +14726,7 @@
         <v>45</v>
       </c>
       <c r="G317" t="s">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="H317" t="s">
         <v>38</v>
@@ -14743,10 +14746,10 @@
         <v>96501.0</v>
       </c>
       <c r="B318" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="C318" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="D318" t="s">
         <v>35</v>
@@ -14758,16 +14761,16 @@
         <v>52</v>
       </c>
       <c r="G318" t="s">
-        <v>1069</v>
+        <v>1070</v>
       </c>
       <c r="H318" t="s">
         <v>38</v>
       </c>
       <c r="I318" t="s">
-        <v>1070</v>
+        <v>1071</v>
       </c>
       <c r="J318" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="K318" t="s">
         <v>2</v>
@@ -14778,10 +14781,10 @@
         <v>94901.0</v>
       </c>
       <c r="B319" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="C319" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
       <c r="D319" t="s">
         <v>35</v>
@@ -14793,16 +14796,16 @@
         <v>45</v>
       </c>
       <c r="G319" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
       <c r="H319" t="s">
         <v>38</v>
       </c>
       <c r="I319" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="J319" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="K319" t="s">
         <v>2</v>
@@ -14813,10 +14816,10 @@
         <v>56102.0</v>
       </c>
       <c r="B320" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="C320" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="D320" t="s">
         <v>35</v>
@@ -14828,13 +14831,13 @@
         <v>45</v>
       </c>
       <c r="G320" t="s">
-        <v>1079</v>
+        <v>1080</v>
       </c>
       <c r="H320" t="s">
         <v>38</v>
       </c>
       <c r="I320" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
       <c r="J320" t="s">
         <v>788</v>
@@ -14869,10 +14872,10 @@
         <v>38</v>
       </c>
       <c r="I321" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="J321" t="s">
-        <v>1080</v>
+        <v>1081</v>
       </c>
       <c r="K321" t="s">
         <v>2</v>
@@ -14883,10 +14886,10 @@
         <v>97401.0</v>
       </c>
       <c r="B322" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
       <c r="C322" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
       <c r="D322" t="s">
         <v>35</v>
@@ -14898,16 +14901,16 @@
         <v>45</v>
       </c>
       <c r="G322" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
       <c r="H322" t="s">
         <v>38</v>
       </c>
       <c r="I322" t="s">
-        <v>1070</v>
+        <v>1071</v>
       </c>
       <c r="J322" t="s">
-        <v>1084</v>
+        <v>1085</v>
       </c>
       <c r="K322" t="s">
         <v>2</v>
@@ -14918,10 +14921,10 @@
         <v>97601.0</v>
       </c>
       <c r="B323" t="s">
-        <v>1085</v>
+        <v>1086</v>
       </c>
       <c r="C323" t="s">
-        <v>1086</v>
+        <v>1087</v>
       </c>
       <c r="D323" t="s">
         <v>839</v>
@@ -14933,13 +14936,13 @@
         <v>45</v>
       </c>
       <c r="G323" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="H323" t="s">
         <v>38</v>
       </c>
       <c r="I323" t="s">
-        <v>1070</v>
+        <v>1071</v>
       </c>
       <c r="J323" t="s">
         <v>841</v>
@@ -14953,10 +14956,10 @@
         <v>53901.0</v>
       </c>
       <c r="B324" t="s">
-        <v>1088</v>
+        <v>1089</v>
       </c>
       <c r="C324" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="D324" t="s">
         <v>43</v>
@@ -14968,7 +14971,7 @@
         <v>139</v>
       </c>
       <c r="G324" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="H324" t="s">
         <v>38</v>
@@ -14988,10 +14991,10 @@
         <v>64002.0</v>
       </c>
       <c r="B325" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="C325" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="D325" t="s">
         <v>70</v>
@@ -15003,16 +15006,16 @@
         <v>45</v>
       </c>
       <c r="G325" t="s">
-        <v>1093</v>
+        <v>1094</v>
       </c>
       <c r="H325" t="s">
         <v>38</v>
       </c>
       <c r="I325" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="J325" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="K325" t="s">
         <v>2</v>
@@ -15023,7 +15026,7 @@
         <v>62701.0</v>
       </c>
       <c r="B326" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="C326" t="s">
         <v>843</v>
@@ -15044,7 +15047,7 @@
         <v>47</v>
       </c>
       <c r="I326" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="J326" t="s">
         <v>49</v>
@@ -15058,7 +15061,7 @@
         <v>63801.0</v>
       </c>
       <c r="B327" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="C327" t="s">
         <v>292</v>
@@ -15073,7 +15076,7 @@
         <v>45</v>
       </c>
       <c r="G327" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="H327" t="s">
         <v>38</v>
@@ -15093,10 +15096,10 @@
         <v>64401.0</v>
       </c>
       <c r="B328" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="C328" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="D328" t="s">
         <v>35</v>
@@ -15108,16 +15111,16 @@
         <v>45</v>
       </c>
       <c r="G328" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="H328" t="s">
         <v>38</v>
       </c>
       <c r="I328" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="J328" t="s">
-        <v>1103</v>
+        <v>1104</v>
       </c>
       <c r="K328" t="s">
         <v>2</v>
@@ -15128,31 +15131,31 @@
         <v>63901.0</v>
       </c>
       <c r="B329" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C329" t="s">
+        <v>1106</v>
+      </c>
+      <c r="D329" t="s">
+        <v>43</v>
+      </c>
+      <c r="E329" t="s">
+        <v>43</v>
+      </c>
+      <c r="F329" t="s">
+        <v>45</v>
+      </c>
+      <c r="G329" t="s">
+        <v>1107</v>
+      </c>
+      <c r="H329" t="s">
+        <v>38</v>
+      </c>
+      <c r="I329" t="s">
+        <v>1095</v>
+      </c>
+      <c r="J329" t="s">
         <v>1104</v>
-      </c>
-      <c r="C329" t="s">
-        <v>1105</v>
-      </c>
-      <c r="D329" t="s">
-        <v>43</v>
-      </c>
-      <c r="E329" t="s">
-        <v>43</v>
-      </c>
-      <c r="F329" t="s">
-        <v>45</v>
-      </c>
-      <c r="G329" t="s">
-        <v>1106</v>
-      </c>
-      <c r="H329" t="s">
-        <v>38</v>
-      </c>
-      <c r="I329" t="s">
-        <v>1094</v>
-      </c>
-      <c r="J329" t="s">
-        <v>1103</v>
       </c>
       <c r="K329" t="s">
         <v>2</v>
@@ -15163,10 +15166,10 @@
         <v>62901.0</v>
       </c>
       <c r="B330" t="s">
-        <v>1107</v>
+        <v>1108</v>
       </c>
       <c r="C330" t="s">
-        <v>1108</v>
+        <v>1109</v>
       </c>
       <c r="D330" t="s">
         <v>43</v>
@@ -15178,13 +15181,13 @@
         <v>45</v>
       </c>
       <c r="G330" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
       <c r="H330" t="s">
         <v>38</v>
       </c>
       <c r="I330" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="J330" t="s">
         <v>948</v>
@@ -15198,10 +15201,10 @@
         <v>61001.0</v>
       </c>
       <c r="B331" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="C331" t="s">
-        <v>1111</v>
+        <v>1112</v>
       </c>
       <c r="D331" t="s">
         <v>44</v>
@@ -15233,10 +15236,10 @@
         <v>61901.0</v>
       </c>
       <c r="B332" t="s">
-        <v>1112</v>
+        <v>1113</v>
       </c>
       <c r="C332" t="s">
-        <v>1113</v>
+        <v>1114</v>
       </c>
       <c r="D332" t="s">
         <v>43</v>
@@ -15248,7 +15251,7 @@
         <v>45</v>
       </c>
       <c r="G332" t="s">
-        <v>1114</v>
+        <v>1115</v>
       </c>
       <c r="H332" t="s">
         <v>38</v>
@@ -15257,7 +15260,7 @@
         <v>254</v>
       </c>
       <c r="J332" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
       <c r="K332" t="s">
         <v>2</v>
@@ -15268,10 +15271,10 @@
         <v>62301.0</v>
       </c>
       <c r="B333" t="s">
-        <v>1116</v>
+        <v>1117</v>
       </c>
       <c r="C333" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="D333" t="s">
         <v>69</v>
@@ -15280,10 +15283,10 @@
         <v>69</v>
       </c>
       <c r="F333" t="s">
-        <v>1118</v>
+        <v>1119</v>
       </c>
       <c r="G333" t="s">
-        <v>1119</v>
+        <v>1120</v>
       </c>
       <c r="H333" t="s">
         <v>38</v>
@@ -15292,7 +15295,7 @@
         <v>410</v>
       </c>
       <c r="J333" t="s">
-        <v>1120</v>
+        <v>1121</v>
       </c>
       <c r="K333" t="s">
         <v>2</v>
@@ -15318,7 +15321,7 @@
         <v>45</v>
       </c>
       <c r="G334" t="s">
-        <v>1121</v>
+        <v>1122</v>
       </c>
       <c r="H334" t="s">
         <v>47</v>
@@ -15338,7 +15341,7 @@
         <v>63401.0</v>
       </c>
       <c r="B335" t="s">
-        <v>1122</v>
+        <v>1123</v>
       </c>
       <c r="C335" t="s">
         <v>305</v>
@@ -15353,7 +15356,7 @@
         <v>45</v>
       </c>
       <c r="G335" t="s">
-        <v>1123</v>
+        <v>1124</v>
       </c>
       <c r="H335" t="s">
         <v>38</v>
@@ -15362,7 +15365,7 @@
         <v>410</v>
       </c>
       <c r="J335" t="s">
-        <v>1124</v>
+        <v>1125</v>
       </c>
       <c r="K335" t="s">
         <v>2</v>
@@ -15373,10 +15376,10 @@
         <v>60501.0</v>
       </c>
       <c r="B336" t="s">
-        <v>1125</v>
+        <v>1126</v>
       </c>
       <c r="C336" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="D336" t="s">
         <v>69</v>
@@ -15388,13 +15391,13 @@
         <v>45</v>
       </c>
       <c r="G336" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="H336" t="s">
         <v>47</v>
       </c>
       <c r="I336" t="s">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="J336" t="s">
         <v>49</v>
@@ -15408,10 +15411,10 @@
         <v>64801.0</v>
       </c>
       <c r="B337" t="s">
-        <v>1129</v>
+        <v>1130</v>
       </c>
       <c r="C337" t="s">
-        <v>1130</v>
+        <v>1131</v>
       </c>
       <c r="D337" t="s">
         <v>43</v>
@@ -15429,10 +15432,10 @@
         <v>38</v>
       </c>
       <c r="I337" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
       <c r="J337" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="K337" t="s">
         <v>2</v>
@@ -15443,31 +15446,31 @@
         <v>68501.0</v>
       </c>
       <c r="B338" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C338" t="s">
+        <v>1135</v>
+      </c>
+      <c r="D338" t="s">
+        <v>43</v>
+      </c>
+      <c r="E338" t="s">
+        <v>43</v>
+      </c>
+      <c r="F338" t="s">
+        <v>1136</v>
+      </c>
+      <c r="G338" t="s">
+        <v>1137</v>
+      </c>
+      <c r="H338" t="s">
+        <v>38</v>
+      </c>
+      <c r="I338" t="s">
+        <v>1132</v>
+      </c>
+      <c r="J338" t="s">
         <v>1133</v>
-      </c>
-      <c r="C338" t="s">
-        <v>1134</v>
-      </c>
-      <c r="D338" t="s">
-        <v>43</v>
-      </c>
-      <c r="E338" t="s">
-        <v>43</v>
-      </c>
-      <c r="F338" t="s">
-        <v>1135</v>
-      </c>
-      <c r="G338" t="s">
-        <v>1136</v>
-      </c>
-      <c r="H338" t="s">
-        <v>38</v>
-      </c>
-      <c r="I338" t="s">
-        <v>1131</v>
-      </c>
-      <c r="J338" t="s">
-        <v>1132</v>
       </c>
       <c r="K338" t="s">
         <v>2</v>
@@ -15478,31 +15481,31 @@
         <v>67301.0</v>
       </c>
       <c r="B339" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C339" t="s">
+        <v>1135</v>
+      </c>
+      <c r="D339" t="s">
+        <v>43</v>
+      </c>
+      <c r="E339" t="s">
+        <v>43</v>
+      </c>
+      <c r="F339" t="s">
+        <v>1136</v>
+      </c>
+      <c r="G339" t="s">
         <v>1137</v>
       </c>
-      <c r="C339" t="s">
-        <v>1134</v>
-      </c>
-      <c r="D339" t="s">
-        <v>43</v>
-      </c>
-      <c r="E339" t="s">
-        <v>43</v>
-      </c>
-      <c r="F339" t="s">
-        <v>1135</v>
-      </c>
-      <c r="G339" t="s">
-        <v>1136</v>
-      </c>
       <c r="H339" t="s">
         <v>38</v>
       </c>
       <c r="I339" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
       <c r="J339" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="K339" t="s">
         <v>2</v>
@@ -15513,10 +15516,10 @@
         <v>66301.0</v>
       </c>
       <c r="B340" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="C340" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="D340" t="s">
         <v>43</v>
@@ -15528,13 +15531,13 @@
         <v>45</v>
       </c>
       <c r="G340" t="s">
-        <v>1140</v>
+        <v>1141</v>
       </c>
       <c r="H340" t="s">
         <v>38</v>
       </c>
       <c r="I340" t="s">
-        <v>1141</v>
+        <v>1142</v>
       </c>
       <c r="J340" t="s">
         <v>432</v>
@@ -15548,10 +15551,10 @@
         <v>67101.0</v>
       </c>
       <c r="B341" t="s">
-        <v>1142</v>
+        <v>1143</v>
       </c>
       <c r="C341" t="s">
-        <v>1143</v>
+        <v>1144</v>
       </c>
       <c r="D341" t="s">
         <v>69</v>
@@ -15563,13 +15566,13 @@
         <v>45</v>
       </c>
       <c r="G341" t="s">
-        <v>1144</v>
+        <v>1145</v>
       </c>
       <c r="H341" t="s">
         <v>47</v>
       </c>
       <c r="I341" t="s">
-        <v>1145</v>
+        <v>1146</v>
       </c>
       <c r="J341" t="s">
         <v>49</v>
@@ -15583,10 +15586,10 @@
         <v>62801.0</v>
       </c>
       <c r="B342" t="s">
-        <v>1146</v>
+        <v>1147</v>
       </c>
       <c r="C342" t="s">
-        <v>1147</v>
+        <v>1148</v>
       </c>
       <c r="D342" t="s">
         <v>69</v>
@@ -15598,16 +15601,16 @@
         <v>52</v>
       </c>
       <c r="G342" t="s">
-        <v>1148</v>
+        <v>1149</v>
       </c>
       <c r="H342" t="s">
         <v>38</v>
       </c>
       <c r="I342" t="s">
-        <v>1149</v>
+        <v>1150</v>
       </c>
       <c r="J342" t="s">
-        <v>1150</v>
+        <v>1151</v>
       </c>
       <c r="K342" t="s">
         <v>2</v>
@@ -15618,10 +15621,10 @@
         <v>64901.0</v>
       </c>
       <c r="B343" t="s">
-        <v>1151</v>
+        <v>1152</v>
       </c>
       <c r="C343" t="s">
-        <v>1152</v>
+        <v>1153</v>
       </c>
       <c r="D343" t="s">
         <v>35</v>
@@ -15633,16 +15636,16 @@
         <v>45</v>
       </c>
       <c r="G343" t="s">
-        <v>1153</v>
+        <v>1154</v>
       </c>
       <c r="H343" t="s">
         <v>38</v>
       </c>
       <c r="I343" t="s">
-        <v>1149</v>
+        <v>1150</v>
       </c>
       <c r="J343" t="s">
-        <v>1150</v>
+        <v>1151</v>
       </c>
       <c r="K343" t="s">
         <v>2</v>
@@ -15653,10 +15656,10 @@
         <v>63501.0</v>
       </c>
       <c r="B344" t="s">
-        <v>1154</v>
+        <v>1155</v>
       </c>
       <c r="C344" t="s">
-        <v>1155</v>
+        <v>1156</v>
       </c>
       <c r="D344" t="s">
         <v>35</v>
@@ -15668,16 +15671,16 @@
         <v>139</v>
       </c>
       <c r="G344" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="H344" t="s">
         <v>38</v>
       </c>
       <c r="I344" t="s">
-        <v>1149</v>
+        <v>1150</v>
       </c>
       <c r="J344" t="s">
-        <v>1157</v>
+        <v>1158</v>
       </c>
       <c r="K344" t="s">
         <v>2</v>
@@ -15688,10 +15691,10 @@
         <v>63701.0</v>
       </c>
       <c r="B345" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="C345" t="s">
-        <v>1159</v>
+        <v>1160</v>
       </c>
       <c r="D345" t="s">
         <v>69</v>
@@ -15703,16 +15706,16 @@
         <v>45</v>
       </c>
       <c r="G345" t="s">
-        <v>1160</v>
+        <v>1161</v>
       </c>
       <c r="H345" t="s">
         <v>38</v>
       </c>
       <c r="I345" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
       <c r="J345" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="K345" t="s">
         <v>2</v>
@@ -15723,7 +15726,7 @@
         <v>68001.0</v>
       </c>
       <c r="B346" t="s">
-        <v>1161</v>
+        <v>1162</v>
       </c>
       <c r="C346" t="s">
         <v>272</v>
@@ -15738,16 +15741,16 @@
         <v>45</v>
       </c>
       <c r="G346" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="H346" t="s">
         <v>38</v>
       </c>
       <c r="I346" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
       <c r="J346" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="K346" t="s">
         <v>2</v>
@@ -15758,10 +15761,10 @@
         <v>64301.0</v>
       </c>
       <c r="B347" t="s">
-        <v>1163</v>
+        <v>1164</v>
       </c>
       <c r="C347" t="s">
-        <v>1164</v>
+        <v>1165</v>
       </c>
       <c r="D347" t="s">
         <v>43</v>
@@ -15773,7 +15776,7 @@
         <v>45</v>
       </c>
       <c r="G347" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="H347" t="s">
         <v>38</v>
@@ -15782,7 +15785,7 @@
         <v>420</v>
       </c>
       <c r="J347" t="s">
-        <v>1166</v>
+        <v>1167</v>
       </c>
       <c r="K347" t="s">
         <v>2</v>
@@ -15793,10 +15796,10 @@
         <v>63301.0</v>
       </c>
       <c r="B348" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="C348" t="s">
-        <v>1168</v>
+        <v>1169</v>
       </c>
       <c r="D348" t="s">
         <v>69</v>
@@ -15814,10 +15817,10 @@
         <v>38</v>
       </c>
       <c r="I348" t="s">
-        <v>1169</v>
+        <v>1170</v>
       </c>
       <c r="J348" t="s">
-        <v>1170</v>
+        <v>1171</v>
       </c>
       <c r="K348" t="s">
         <v>2</v>
@@ -15828,10 +15831,10 @@
         <v>68201.0</v>
       </c>
       <c r="B349" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="C349" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="D349" t="s">
         <v>43</v>
@@ -15843,16 +15846,16 @@
         <v>139</v>
       </c>
       <c r="G349" t="s">
-        <v>1173</v>
+        <v>1174</v>
       </c>
       <c r="H349" t="s">
         <v>38</v>
       </c>
       <c r="I349" t="s">
-        <v>1174</v>
+        <v>1175</v>
       </c>
       <c r="J349" t="s">
-        <v>1175</v>
+        <v>1176</v>
       </c>
       <c r="K349" t="s">
         <v>2</v>
@@ -15863,10 +15866,10 @@
         <v>58201.0</v>
       </c>
       <c r="B350" t="s">
-        <v>1176</v>
+        <v>1177</v>
       </c>
       <c r="C350" t="s">
-        <v>1177</v>
+        <v>1178</v>
       </c>
       <c r="D350" t="s">
         <v>69</v>
@@ -15878,7 +15881,7 @@
         <v>45</v>
       </c>
       <c r="G350" t="s">
-        <v>1178</v>
+        <v>1179</v>
       </c>
       <c r="H350" t="s">
         <v>38</v>
@@ -15887,7 +15890,7 @@
         <v>136</v>
       </c>
       <c r="J350" t="s">
-        <v>1179</v>
+        <v>1180</v>
       </c>
       <c r="K350" t="s">
         <v>2</v>
@@ -15898,10 +15901,10 @@
         <v>56101.0</v>
       </c>
       <c r="B351" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="C351" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="D351" t="s">
         <v>35</v>
@@ -15913,7 +15916,7 @@
         <v>45</v>
       </c>
       <c r="G351" t="s">
-        <v>1180</v>
+        <v>1181</v>
       </c>
       <c r="H351" t="s">
         <v>38</v>
@@ -15922,7 +15925,7 @@
         <v>376</v>
       </c>
       <c r="J351" t="s">
-        <v>1181</v>
+        <v>1182</v>
       </c>
       <c r="K351" t="s">
         <v>2</v>
@@ -15933,10 +15936,10 @@
         <v>57201.0</v>
       </c>
       <c r="B352" t="s">
-        <v>1182</v>
+        <v>1183</v>
       </c>
       <c r="C352" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="D352" t="s">
         <v>70</v>
@@ -15948,7 +15951,7 @@
         <v>45</v>
       </c>
       <c r="G352" t="s">
-        <v>1183</v>
+        <v>1184</v>
       </c>
       <c r="H352" t="s">
         <v>38</v>
@@ -15957,7 +15960,7 @@
         <v>376</v>
       </c>
       <c r="J352" t="s">
-        <v>1184</v>
+        <v>1185</v>
       </c>
       <c r="K352" t="s">
         <v>2</v>
@@ -15968,7 +15971,7 @@
         <v>52801.0</v>
       </c>
       <c r="B353" t="s">
-        <v>1185</v>
+        <v>1186</v>
       </c>
       <c r="C353" t="s">
         <v>323</v>
@@ -15983,7 +15986,7 @@
         <v>45</v>
       </c>
       <c r="G353" t="s">
-        <v>1186</v>
+        <v>1187</v>
       </c>
       <c r="H353" t="s">
         <v>38</v>
@@ -15992,7 +15995,7 @@
         <v>136</v>
       </c>
       <c r="J353" t="s">
-        <v>1179</v>
+        <v>1180</v>
       </c>
       <c r="K353" t="s">
         <v>2</v>
@@ -16003,10 +16006,10 @@
         <v>55401.0</v>
       </c>
       <c r="B354" t="s">
-        <v>1187</v>
+        <v>1188</v>
       </c>
       <c r="C354" t="s">
-        <v>1188</v>
+        <v>1189</v>
       </c>
       <c r="D354" t="s">
         <v>69</v>
@@ -16018,7 +16021,7 @@
         <v>45</v>
       </c>
       <c r="G354" t="s">
-        <v>1189</v>
+        <v>1190</v>
       </c>
       <c r="H354" t="s">
         <v>38</v>
@@ -16027,7 +16030,7 @@
         <v>348</v>
       </c>
       <c r="J354" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
       <c r="K354" t="s">
         <v>2</v>
@@ -16038,10 +16041,10 @@
         <v>58101.0</v>
       </c>
       <c r="B355" t="s">
-        <v>1191</v>
+        <v>1192</v>
       </c>
       <c r="C355" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="D355" t="s">
         <v>69</v>
@@ -16053,7 +16056,7 @@
         <v>45</v>
       </c>
       <c r="G355" t="s">
-        <v>1193</v>
+        <v>1194</v>
       </c>
       <c r="H355" t="s">
         <v>38</v>
@@ -16062,7 +16065,7 @@
         <v>348</v>
       </c>
       <c r="J355" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="K355" t="s">
         <v>2</v>
@@ -16073,10 +16076,10 @@
         <v>54401.0</v>
       </c>
       <c r="B356" t="s">
-        <v>1195</v>
+        <v>1196</v>
       </c>
       <c r="C356" t="s">
-        <v>1196</v>
+        <v>1197</v>
       </c>
       <c r="D356" t="s">
         <v>43</v>
@@ -16088,7 +16091,7 @@
         <v>45</v>
       </c>
       <c r="G356" t="s">
-        <v>1197</v>
+        <v>1198</v>
       </c>
       <c r="H356" t="s">
         <v>38</v>
@@ -16097,7 +16100,7 @@
         <v>106</v>
       </c>
       <c r="J356" t="s">
-        <v>1198</v>
+        <v>1199</v>
       </c>
       <c r="K356" t="s">
         <v>2</v>
@@ -16108,10 +16111,10 @@
         <v>52601.0</v>
       </c>
       <c r="B357" t="s">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="C357" t="s">
-        <v>1200</v>
+        <v>1201</v>
       </c>
       <c r="D357" t="s">
         <v>35</v>
@@ -16123,7 +16126,7 @@
         <v>45</v>
       </c>
       <c r="G357" t="s">
-        <v>1201</v>
+        <v>1202</v>
       </c>
       <c r="H357" t="s">
         <v>38</v>
@@ -16132,7 +16135,7 @@
         <v>125</v>
       </c>
       <c r="J357" t="s">
-        <v>1202</v>
+        <v>1203</v>
       </c>
       <c r="K357" t="s">
         <v>2</v>
@@ -16143,7 +16146,7 @@
         <v>56501.0</v>
       </c>
       <c r="B358" t="s">
-        <v>1203</v>
+        <v>1204</v>
       </c>
       <c r="C358" t="s">
         <v>191</v>
@@ -16158,16 +16161,16 @@
         <v>45</v>
       </c>
       <c r="G358" t="s">
-        <v>1204</v>
+        <v>1205</v>
       </c>
       <c r="H358" t="s">
         <v>38</v>
       </c>
       <c r="I358" t="s">
-        <v>1205</v>
+        <v>1206</v>
       </c>
       <c r="J358" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="K358" t="s">
         <v>2</v>
@@ -16178,10 +16181,10 @@
         <v>55301.0</v>
       </c>
       <c r="B359" t="s">
-        <v>1207</v>
+        <v>1208</v>
       </c>
       <c r="C359" t="s">
-        <v>1208</v>
+        <v>1209</v>
       </c>
       <c r="D359" t="s">
         <v>35</v>
@@ -16202,7 +16205,7 @@
         <v>103</v>
       </c>
       <c r="J359" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="K359" t="s">
         <v>2</v>
@@ -16213,10 +16216,10 @@
         <v>55501.0</v>
       </c>
       <c r="B360" t="s">
-        <v>1209</v>
+        <v>1210</v>
       </c>
       <c r="C360" t="s">
-        <v>1210</v>
+        <v>1211</v>
       </c>
       <c r="D360" t="s">
         <v>43</v>
@@ -16228,7 +16231,7 @@
         <v>45</v>
       </c>
       <c r="G360" t="s">
-        <v>1211</v>
+        <v>1212</v>
       </c>
       <c r="H360" t="s">
         <v>38</v>
@@ -16237,7 +16240,7 @@
         <v>114</v>
       </c>
       <c r="J360" t="s">
-        <v>1212</v>
+        <v>1213</v>
       </c>
       <c r="K360" t="s">
         <v>2</v>
@@ -16248,10 +16251,10 @@
         <v>61401.0</v>
       </c>
       <c r="B361" t="s">
-        <v>1213</v>
+        <v>1214</v>
       </c>
       <c r="C361" t="s">
-        <v>1214</v>
+        <v>1215</v>
       </c>
       <c r="D361" t="s">
         <v>43</v>
@@ -16263,16 +16266,16 @@
         <v>45</v>
       </c>
       <c r="G361" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="H361" t="s">
         <v>38</v>
       </c>
       <c r="I361" t="s">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="J361" t="s">
-        <v>1215</v>
+        <v>1216</v>
       </c>
       <c r="K361" t="s">
         <v>2</v>
@@ -16283,7 +16286,7 @@
         <v>54801.0</v>
       </c>
       <c r="B362" t="s">
-        <v>1216</v>
+        <v>1217</v>
       </c>
       <c r="C362" t="s">
         <v>877</v>
@@ -16298,13 +16301,13 @@
         <v>45</v>
       </c>
       <c r="G362" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="H362" t="s">
         <v>47</v>
       </c>
       <c r="I362" t="s">
-        <v>1217</v>
+        <v>1218</v>
       </c>
       <c r="J362" t="s">
         <v>49</v>
@@ -16318,10 +16321,10 @@
         <v>60301.0</v>
       </c>
       <c r="B363" t="s">
-        <v>1218</v>
+        <v>1219</v>
       </c>
       <c r="C363" t="s">
-        <v>1177</v>
+        <v>1178</v>
       </c>
       <c r="D363" t="s">
         <v>69</v>
@@ -16333,13 +16336,13 @@
         <v>45</v>
       </c>
       <c r="G363" t="s">
-        <v>1219</v>
+        <v>1220</v>
       </c>
       <c r="H363" t="s">
         <v>47</v>
       </c>
       <c r="I363" t="s">
-        <v>1220</v>
+        <v>1221</v>
       </c>
       <c r="J363" t="s">
         <v>49</v>
@@ -16353,10 +16356,10 @@
         <v>59401.0</v>
       </c>
       <c r="B364" t="s">
-        <v>1221</v>
+        <v>1222</v>
       </c>
       <c r="C364" t="s">
-        <v>1222</v>
+        <v>1223</v>
       </c>
       <c r="D364" t="s">
         <v>69</v>
@@ -16368,13 +16371,13 @@
         <v>45</v>
       </c>
       <c r="G364" t="s">
-        <v>1223</v>
+        <v>1224</v>
       </c>
       <c r="H364" t="s">
         <v>38</v>
       </c>
       <c r="I364" t="s">
-        <v>1224</v>
+        <v>1225</v>
       </c>
       <c r="J364" t="s">
         <v>714</v>
@@ -16388,7 +16391,7 @@
         <v>54802.0</v>
       </c>
       <c r="B365" t="s">
-        <v>1216</v>
+        <v>1217</v>
       </c>
       <c r="C365" t="s">
         <v>877</v>
@@ -16403,16 +16406,16 @@
         <v>45</v>
       </c>
       <c r="G365" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="H365" t="s">
         <v>38</v>
       </c>
       <c r="I365" t="s">
-        <v>1217</v>
+        <v>1218</v>
       </c>
       <c r="J365" t="s">
-        <v>1225</v>
+        <v>1226</v>
       </c>
       <c r="K365" t="s">
         <v>2</v>
@@ -16423,10 +16426,10 @@
         <v>57101.0</v>
       </c>
       <c r="B366" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C366" t="s">
-        <v>1227</v>
+        <v>1228</v>
       </c>
       <c r="D366" t="s">
         <v>35</v>
@@ -16438,7 +16441,7 @@
         <v>45</v>
       </c>
       <c r="G366" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
       <c r="H366" t="s">
         <v>38</v>
@@ -16447,7 +16450,7 @@
         <v>393</v>
       </c>
       <c r="J366" t="s">
-        <v>1229</v>
+        <v>1230</v>
       </c>
       <c r="K366" t="s">
         <v>2</v>
@@ -16458,10 +16461,10 @@
         <v>56901.0</v>
       </c>
       <c r="B367" t="s">
-        <v>1230</v>
+        <v>1231</v>
       </c>
       <c r="C367" t="s">
-        <v>1231</v>
+        <v>1232</v>
       </c>
       <c r="D367" t="s">
         <v>69</v>
@@ -16473,16 +16476,16 @@
         <v>45</v>
       </c>
       <c r="G367" t="s">
-        <v>1232</v>
+        <v>1233</v>
       </c>
       <c r="H367" t="s">
         <v>38</v>
       </c>
       <c r="I367" t="s">
-        <v>1233</v>
+        <v>1234</v>
       </c>
       <c r="J367" t="s">
-        <v>1234</v>
+        <v>1235</v>
       </c>
       <c r="K367" t="s">
         <v>2</v>
@@ -16493,10 +16496,10 @@
         <v>58901.0</v>
       </c>
       <c r="B368" t="s">
-        <v>1235</v>
+        <v>1236</v>
       </c>
       <c r="C368" t="s">
-        <v>1236</v>
+        <v>1237</v>
       </c>
       <c r="D368" t="s">
         <v>35</v>
@@ -16508,16 +16511,16 @@
         <v>45</v>
       </c>
       <c r="G368" t="s">
-        <v>1237</v>
+        <v>1238</v>
       </c>
       <c r="H368" t="s">
         <v>38</v>
       </c>
       <c r="I368" t="s">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="J368" t="s">
-        <v>1239</v>
+        <v>1240</v>
       </c>
       <c r="K368" t="s">
         <v>2</v>
@@ -16528,10 +16531,10 @@
         <v>56801.0</v>
       </c>
       <c r="B369" t="s">
-        <v>1240</v>
+        <v>1241</v>
       </c>
       <c r="C369" t="s">
-        <v>1241</v>
+        <v>1242</v>
       </c>
       <c r="D369" t="s">
         <v>35</v>
@@ -16543,16 +16546,16 @@
         <v>45</v>
       </c>
       <c r="G369" t="s">
-        <v>1242</v>
+        <v>1243</v>
       </c>
       <c r="H369" t="s">
         <v>38</v>
       </c>
       <c r="I369" t="s">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="J369" t="s">
-        <v>1243</v>
+        <v>1244</v>
       </c>
       <c r="K369" t="s">
         <v>2</v>
@@ -16563,10 +16566,10 @@
         <v>59601.0</v>
       </c>
       <c r="B370" t="s">
-        <v>1244</v>
+        <v>1245</v>
       </c>
       <c r="C370" t="s">
-        <v>1222</v>
+        <v>1223</v>
       </c>
       <c r="D370" t="s">
         <v>35</v>
@@ -16578,13 +16581,13 @@
         <v>45</v>
       </c>
       <c r="G370" t="s">
-        <v>1223</v>
+        <v>1224</v>
       </c>
       <c r="H370" t="s">
         <v>38</v>
       </c>
       <c r="I370" t="s">
-        <v>1224</v>
+        <v>1225</v>
       </c>
       <c r="J370" t="s">
         <v>714</v>
@@ -16598,7 +16601,7 @@
         <v>59901.0</v>
       </c>
       <c r="B371" t="s">
-        <v>1245</v>
+        <v>1246</v>
       </c>
       <c r="C371" t="s">
         <v>68</v>
@@ -16613,16 +16616,16 @@
         <v>45</v>
       </c>
       <c r="G371" t="s">
-        <v>1246</v>
+        <v>1247</v>
       </c>
       <c r="H371" t="s">
         <v>38</v>
       </c>
       <c r="I371" t="s">
-        <v>1247</v>
+        <v>1248</v>
       </c>
       <c r="J371" t="s">
-        <v>1248</v>
+        <v>1249</v>
       </c>
       <c r="K371" t="s">
         <v>2</v>
@@ -16633,7 +16636,7 @@
         <v>57701.0</v>
       </c>
       <c r="B372" t="s">
-        <v>1249</v>
+        <v>1250</v>
       </c>
       <c r="C372" t="s">
         <v>880</v>
@@ -16648,16 +16651,16 @@
         <v>45</v>
       </c>
       <c r="G372" t="s">
-        <v>1250</v>
+        <v>1251</v>
       </c>
       <c r="H372" t="s">
         <v>38</v>
       </c>
       <c r="I372" t="s">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="J372" t="s">
-        <v>1251</v>
+        <v>1252</v>
       </c>
       <c r="K372" t="s">
         <v>2</v>
@@ -16668,10 +16671,10 @@
         <v>59501.0</v>
       </c>
       <c r="B373" t="s">
-        <v>1252</v>
+        <v>1253</v>
       </c>
       <c r="C373" t="s">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="D373" t="s">
         <v>43</v>
@@ -16683,16 +16686,16 @@
         <v>45</v>
       </c>
       <c r="G373" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="H373" t="s">
         <v>38</v>
       </c>
       <c r="I373" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="J373" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
       <c r="K373" t="s">
         <v>2</v>
@@ -16703,10 +16706,10 @@
         <v>79701.0</v>
       </c>
       <c r="B374" t="s">
-        <v>1257</v>
+        <v>1258</v>
       </c>
       <c r="C374" t="s">
-        <v>1258</v>
+        <v>1259</v>
       </c>
       <c r="D374" t="s">
         <v>43</v>
@@ -16718,7 +16721,7 @@
         <v>139</v>
       </c>
       <c r="G374" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="H374" t="s">
         <v>38</v>
@@ -16727,7 +16730,7 @@
         <v>553</v>
       </c>
       <c r="J374" t="s">
-        <v>1260</v>
+        <v>1261</v>
       </c>
       <c r="K374" t="s">
         <v>2</v>
@@ -16738,10 +16741,10 @@
         <v>78101.0</v>
       </c>
       <c r="B375" t="s">
-        <v>1261</v>
+        <v>1262</v>
       </c>
       <c r="C375" t="s">
-        <v>1241</v>
+        <v>1242</v>
       </c>
       <c r="D375" t="s">
         <v>35</v>
@@ -16753,13 +16756,13 @@
         <v>45</v>
       </c>
       <c r="G375" t="s">
-        <v>1262</v>
+        <v>1263</v>
       </c>
       <c r="H375" t="s">
         <v>38</v>
       </c>
       <c r="I375" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="J375" t="s">
         <v>740</v>
@@ -16773,7 +16776,7 @@
         <v>78001.0</v>
       </c>
       <c r="B376" t="s">
-        <v>1264</v>
+        <v>1265</v>
       </c>
       <c r="C376" t="s">
         <v>571</v>
@@ -16788,7 +16791,7 @@
         <v>45</v>
       </c>
       <c r="G376" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
       <c r="H376" t="s">
         <v>38</v>
@@ -16808,7 +16811,7 @@
         <v>77701.0</v>
       </c>
       <c r="B377" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="C377" t="s">
         <v>716</v>
@@ -16823,13 +16826,13 @@
         <v>45</v>
       </c>
       <c r="G377" t="s">
-        <v>1267</v>
+        <v>1268</v>
       </c>
       <c r="H377" t="s">
         <v>38</v>
       </c>
       <c r="I377" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="J377" t="s">
         <v>787</v>
@@ -16843,10 +16846,10 @@
         <v>78401.0</v>
       </c>
       <c r="B378" t="s">
-        <v>1269</v>
+        <v>1270</v>
       </c>
       <c r="C378" t="s">
-        <v>1270</v>
+        <v>1271</v>
       </c>
       <c r="D378" t="s">
         <v>533</v>
@@ -16858,13 +16861,13 @@
         <v>45</v>
       </c>
       <c r="G378" t="s">
-        <v>1271</v>
+        <v>1272</v>
       </c>
       <c r="H378" t="s">
         <v>38</v>
       </c>
       <c r="I378" t="s">
-        <v>1272</v>
+        <v>1273</v>
       </c>
       <c r="J378" t="s">
         <v>513</v>
@@ -16878,10 +16881,10 @@
         <v>78901.0</v>
       </c>
       <c r="B379" t="s">
-        <v>1273</v>
+        <v>1274</v>
       </c>
       <c r="C379" t="s">
-        <v>1274</v>
+        <v>1275</v>
       </c>
       <c r="D379" t="s">
         <v>69</v>
@@ -16893,13 +16896,13 @@
         <v>45</v>
       </c>
       <c r="G379" t="s">
-        <v>1275</v>
+        <v>1276</v>
       </c>
       <c r="H379" t="s">
         <v>38</v>
       </c>
       <c r="I379" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
       <c r="J379" t="s">
         <v>801</v>
@@ -16913,10 +16916,10 @@
         <v>73202.0</v>
       </c>
       <c r="B380" t="s">
-        <v>1276</v>
+        <v>1277</v>
       </c>
       <c r="C380" t="s">
-        <v>1277</v>
+        <v>1278</v>
       </c>
       <c r="D380" t="s">
         <v>35</v>
@@ -16928,13 +16931,13 @@
         <v>45</v>
       </c>
       <c r="G380" t="s">
-        <v>1278</v>
+        <v>1279</v>
       </c>
       <c r="H380" t="s">
         <v>38</v>
       </c>
       <c r="I380" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
       <c r="J380" t="s">
         <v>801</v>
@@ -16948,10 +16951,10 @@
         <v>76601.0</v>
       </c>
       <c r="B381" t="s">
-        <v>1279</v>
+        <v>1280</v>
       </c>
       <c r="C381" t="s">
-        <v>1280</v>
+        <v>1281</v>
       </c>
       <c r="D381" t="s">
         <v>43</v>
@@ -16963,16 +16966,16 @@
         <v>139</v>
       </c>
       <c r="G381" t="s">
-        <v>1281</v>
+        <v>1282</v>
       </c>
       <c r="H381" t="s">
         <v>38</v>
       </c>
       <c r="I381" t="s">
-        <v>1282</v>
+        <v>1283</v>
       </c>
       <c r="J381" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
       <c r="K381" t="s">
         <v>2</v>
@@ -16983,7 +16986,7 @@
         <v>75301.0</v>
       </c>
       <c r="B382" t="s">
-        <v>1284</v>
+        <v>1285</v>
       </c>
       <c r="C382" t="s">
         <v>790</v>
@@ -16998,13 +17001,13 @@
         <v>45</v>
       </c>
       <c r="G382" t="s">
-        <v>1285</v>
+        <v>1286</v>
       </c>
       <c r="H382" t="s">
         <v>47</v>
       </c>
       <c r="I382" t="s">
-        <v>1282</v>
+        <v>1283</v>
       </c>
       <c r="J382" t="s">
         <v>49</v>
@@ -17018,7 +17021,7 @@
         <v>76901.0</v>
       </c>
       <c r="B383" t="s">
-        <v>1286</v>
+        <v>1287</v>
       </c>
       <c r="C383" t="s">
         <v>790</v>
@@ -17033,16 +17036,16 @@
         <v>45</v>
       </c>
       <c r="G383" t="s">
-        <v>1287</v>
+        <v>1288</v>
       </c>
       <c r="H383" t="s">
         <v>38</v>
       </c>
       <c r="I383" t="s">
-        <v>1215</v>
+        <v>1216</v>
       </c>
       <c r="J383" t="s">
-        <v>1288</v>
+        <v>1289</v>
       </c>
       <c r="K383" t="s">
         <v>2</v>
@@ -17053,10 +17056,10 @@
         <v>77101.0</v>
       </c>
       <c r="B384" t="s">
-        <v>1289</v>
+        <v>1290</v>
       </c>
       <c r="C384" t="s">
-        <v>1290</v>
+        <v>1291</v>
       </c>
       <c r="D384" t="s">
         <v>44</v>
@@ -17068,13 +17071,13 @@
         <v>45</v>
       </c>
       <c r="G384" t="s">
-        <v>1291</v>
+        <v>1292</v>
       </c>
       <c r="H384" t="s">
         <v>38</v>
       </c>
       <c r="I384" t="s">
-        <v>1229</v>
+        <v>1230</v>
       </c>
       <c r="J384" t="s">
         <v>964</v>
@@ -17088,7 +17091,7 @@
         <v>77201.0</v>
       </c>
       <c r="B385" t="s">
-        <v>1292</v>
+        <v>1293</v>
       </c>
       <c r="C385" t="s">
         <v>658</v>
@@ -17109,7 +17112,7 @@
         <v>38</v>
       </c>
       <c r="I385" t="s">
-        <v>1229</v>
+        <v>1230</v>
       </c>
       <c r="J385" t="s">
         <v>792</v>
@@ -17123,10 +17126,10 @@
         <v>76501.0</v>
       </c>
       <c r="B386" t="s">
-        <v>1293</v>
+        <v>1294</v>
       </c>
       <c r="C386" t="s">
-        <v>1294</v>
+        <v>1295</v>
       </c>
       <c r="D386" t="s">
         <v>43</v>
@@ -17138,16 +17141,16 @@
         <v>45</v>
       </c>
       <c r="G386" t="s">
-        <v>1295</v>
+        <v>1296</v>
       </c>
       <c r="H386" t="s">
         <v>38</v>
       </c>
       <c r="I386" t="s">
-        <v>1225</v>
+        <v>1226</v>
       </c>
       <c r="J386" t="s">
-        <v>1296</v>
+        <v>1297</v>
       </c>
       <c r="K386" t="s">
         <v>2</v>
@@ -17158,10 +17161,10 @@
         <v>79601.0</v>
       </c>
       <c r="B387" t="s">
-        <v>1297</v>
+        <v>1298</v>
       </c>
       <c r="C387" t="s">
-        <v>1298</v>
+        <v>1299</v>
       </c>
       <c r="D387" t="s">
         <v>69</v>
@@ -17173,16 +17176,16 @@
         <v>45</v>
       </c>
       <c r="G387" t="s">
-        <v>1299</v>
+        <v>1300</v>
       </c>
       <c r="H387" t="s">
         <v>38</v>
       </c>
       <c r="I387" t="s">
-        <v>1300</v>
+        <v>1301</v>
       </c>
       <c r="J387" t="s">
-        <v>1301</v>
+        <v>1302</v>
       </c>
       <c r="K387" t="s">
         <v>2</v>
@@ -17193,7 +17196,7 @@
         <v>81501.0</v>
       </c>
       <c r="B388" t="s">
-        <v>1302</v>
+        <v>1303</v>
       </c>
       <c r="C388" t="s">
         <v>765</v>
@@ -17214,10 +17217,10 @@
         <v>38</v>
       </c>
       <c r="I388" t="s">
-        <v>1300</v>
+        <v>1301</v>
       </c>
       <c r="J388" t="s">
-        <v>1301</v>
+        <v>1302</v>
       </c>
       <c r="K388" t="s">
         <v>2</v>
@@ -17228,10 +17231,10 @@
         <v>81001.0</v>
       </c>
       <c r="B389" t="s">
-        <v>1303</v>
+        <v>1304</v>
       </c>
       <c r="C389" t="s">
-        <v>1304</v>
+        <v>1305</v>
       </c>
       <c r="D389" t="s">
         <v>69</v>
@@ -17243,16 +17246,16 @@
         <v>52</v>
       </c>
       <c r="G389" t="s">
-        <v>1305</v>
+        <v>1306</v>
       </c>
       <c r="H389" t="s">
         <v>38</v>
       </c>
       <c r="I389" t="s">
-        <v>1300</v>
+        <v>1301</v>
       </c>
       <c r="J389" t="s">
-        <v>1301</v>
+        <v>1302</v>
       </c>
       <c r="K389" t="s">
         <v>2</v>
@@ -17284,10 +17287,10 @@
         <v>38</v>
       </c>
       <c r="I390" t="s">
-        <v>1166</v>
+        <v>1167</v>
       </c>
       <c r="J390" t="s">
-        <v>1306</v>
+        <v>1307</v>
       </c>
       <c r="K390" t="s">
         <v>2</v>
@@ -17298,10 +17301,10 @@
         <v>82001.0</v>
       </c>
       <c r="B391" t="s">
-        <v>1307</v>
+        <v>1308</v>
       </c>
       <c r="C391" t="s">
-        <v>1196</v>
+        <v>1197</v>
       </c>
       <c r="D391" t="s">
         <v>43</v>
@@ -17313,7 +17316,7 @@
         <v>45</v>
       </c>
       <c r="G391" t="s">
-        <v>1308</v>
+        <v>1309</v>
       </c>
       <c r="H391" t="s">
         <v>38</v>
@@ -17322,7 +17325,7 @@
         <v>553</v>
       </c>
       <c r="J391" t="s">
-        <v>1309</v>
+        <v>1310</v>
       </c>
       <c r="K391" t="s">
         <v>2</v>
@@ -17333,10 +17336,10 @@
         <v>78301.0</v>
       </c>
       <c r="B392" t="s">
-        <v>1310</v>
+        <v>1311</v>
       </c>
       <c r="C392" t="s">
-        <v>1311</v>
+        <v>1312</v>
       </c>
       <c r="D392" t="s">
         <v>69</v>
@@ -17348,7 +17351,7 @@
         <v>45</v>
       </c>
       <c r="G392" t="s">
-        <v>1312</v>
+        <v>1313</v>
       </c>
       <c r="H392" t="s">
         <v>38</v>
@@ -17357,7 +17360,7 @@
         <v>575</v>
       </c>
       <c r="J392" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
       <c r="K392" t="s">
         <v>2</v>
@@ -17383,16 +17386,16 @@
         <v>52</v>
       </c>
       <c r="G393" t="s">
-        <v>1313</v>
+        <v>1314</v>
       </c>
       <c r="H393" t="s">
         <v>38</v>
       </c>
       <c r="I393" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="J393" t="s">
-        <v>1314</v>
+        <v>1315</v>
       </c>
       <c r="K393" t="s">
         <v>2</v>
@@ -17403,10 +17406,10 @@
         <v>79101.0</v>
       </c>
       <c r="B394" t="s">
-        <v>1315</v>
+        <v>1316</v>
       </c>
       <c r="C394" t="s">
-        <v>1113</v>
+        <v>1114</v>
       </c>
       <c r="D394" t="s">
         <v>70</v>
@@ -17418,16 +17421,16 @@
         <v>45</v>
       </c>
       <c r="G394" t="s">
-        <v>1316</v>
+        <v>1317</v>
       </c>
       <c r="H394" t="s">
         <v>38</v>
       </c>
       <c r="I394" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="J394" t="s">
-        <v>1314</v>
+        <v>1315</v>
       </c>
       <c r="K394" t="s">
         <v>2</v>
@@ -17438,10 +17441,10 @@
         <v>81101.0</v>
       </c>
       <c r="B395" t="s">
-        <v>1317</v>
+        <v>1318</v>
       </c>
       <c r="C395" t="s">
-        <v>1168</v>
+        <v>1169</v>
       </c>
       <c r="D395" t="s">
         <v>70</v>
@@ -17453,16 +17456,16 @@
         <v>45</v>
       </c>
       <c r="G395" t="s">
-        <v>1318</v>
+        <v>1319</v>
       </c>
       <c r="H395" t="s">
         <v>38</v>
       </c>
       <c r="I395" t="s">
-        <v>1300</v>
+        <v>1301</v>
       </c>
       <c r="J395" t="s">
-        <v>1282</v>
+        <v>1283</v>
       </c>
       <c r="K395" t="s">
         <v>2</v>
@@ -17473,10 +17476,10 @@
         <v>80901.0</v>
       </c>
       <c r="B396" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
       <c r="C396" t="s">
-        <v>1320</v>
+        <v>1321</v>
       </c>
       <c r="D396" t="s">
         <v>43</v>
@@ -17488,13 +17491,13 @@
         <v>45</v>
       </c>
       <c r="G396" t="s">
-        <v>1321</v>
+        <v>1322</v>
       </c>
       <c r="H396" t="s">
         <v>38</v>
       </c>
       <c r="I396" t="s">
-        <v>1322</v>
+        <v>1323</v>
       </c>
       <c r="J396" t="s">
         <v>772</v>
@@ -17508,7 +17511,7 @@
         <v>80201.0</v>
       </c>
       <c r="B397" t="s">
-        <v>1323</v>
+        <v>1324</v>
       </c>
       <c r="C397" t="s">
         <v>264</v>
@@ -17529,10 +17532,10 @@
         <v>38</v>
       </c>
       <c r="I397" t="s">
-        <v>1150</v>
+        <v>1151</v>
       </c>
       <c r="J397" t="s">
-        <v>1324</v>
+        <v>1325</v>
       </c>
       <c r="K397" t="s">
         <v>2</v>
@@ -17543,10 +17546,10 @@
         <v>80801.0</v>
       </c>
       <c r="B398" t="s">
-        <v>1325</v>
+        <v>1326</v>
       </c>
       <c r="C398" t="s">
-        <v>1326</v>
+        <v>1327</v>
       </c>
       <c r="D398" t="s">
         <v>43</v>
@@ -17558,13 +17561,13 @@
         <v>45</v>
       </c>
       <c r="G398" t="s">
-        <v>1327</v>
+        <v>1328</v>
       </c>
       <c r="H398" t="s">
         <v>38</v>
       </c>
       <c r="I398" t="s">
-        <v>1328</v>
+        <v>1329</v>
       </c>
       <c r="J398" t="s">
         <v>586</v>
@@ -17578,10 +17581,10 @@
         <v>69801.0</v>
       </c>
       <c r="B399" t="s">
-        <v>1329</v>
+        <v>1330</v>
       </c>
       <c r="C399" t="s">
-        <v>1330</v>
+        <v>1331</v>
       </c>
       <c r="D399" t="s">
         <v>44</v>
@@ -17599,10 +17602,10 @@
         <v>38</v>
       </c>
       <c r="I399" t="s">
-        <v>1331</v>
+        <v>1332</v>
       </c>
       <c r="J399" t="s">
-        <v>1332</v>
+        <v>1333</v>
       </c>
       <c r="K399" t="s">
         <v>2</v>
@@ -17613,10 +17616,10 @@
         <v>70601.0</v>
       </c>
       <c r="B400" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="C400" t="s">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="D400" t="s">
         <v>43</v>
@@ -17648,10 +17651,10 @@
         <v>67001.0</v>
       </c>
       <c r="B401" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="C401" t="s">
-        <v>1336</v>
+        <v>1337</v>
       </c>
       <c r="D401" t="s">
         <v>35</v>
@@ -17663,16 +17666,16 @@
         <v>45</v>
       </c>
       <c r="G401" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="H401" t="s">
         <v>38</v>
       </c>
       <c r="I401" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="J401" t="s">
-        <v>1339</v>
+        <v>1340</v>
       </c>
       <c r="K401" t="s">
         <v>2</v>
@@ -17683,10 +17686,10 @@
         <v>70301.0</v>
       </c>
       <c r="B402" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="C402" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="D402" t="s">
         <v>43</v>
@@ -17698,13 +17701,13 @@
         <v>45</v>
       </c>
       <c r="G402" t="s">
-        <v>1342</v>
+        <v>1343</v>
       </c>
       <c r="H402" t="s">
         <v>38</v>
       </c>
       <c r="I402" t="s">
-        <v>1343</v>
+        <v>1344</v>
       </c>
       <c r="J402" t="s">
         <v>500</v>
@@ -17718,10 +17721,10 @@
         <v>71701.0</v>
       </c>
       <c r="B403" t="s">
-        <v>1344</v>
+        <v>1345</v>
       </c>
       <c r="C403" t="s">
-        <v>1345</v>
+        <v>1346</v>
       </c>
       <c r="D403" t="s">
         <v>35</v>
@@ -17753,10 +17756,10 @@
         <v>70901.0</v>
       </c>
       <c r="B404" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="C404" t="s">
-        <v>1143</v>
+        <v>1144</v>
       </c>
       <c r="D404" t="s">
         <v>69</v>
@@ -17768,7 +17771,7 @@
         <v>45</v>
       </c>
       <c r="G404" t="s">
-        <v>1347</v>
+        <v>1348</v>
       </c>
       <c r="H404" t="s">
         <v>47</v>
@@ -17788,7 +17791,7 @@
         <v>71601.0</v>
       </c>
       <c r="B405" t="s">
-        <v>1348</v>
+        <v>1349</v>
       </c>
       <c r="C405" t="s">
         <v>100</v>
@@ -17803,7 +17806,7 @@
         <v>45</v>
       </c>
       <c r="G405" t="s">
-        <v>1349</v>
+        <v>1350</v>
       </c>
       <c r="H405" t="s">
         <v>38</v>
@@ -17823,10 +17826,10 @@
         <v>70101.0</v>
       </c>
       <c r="B406" t="s">
-        <v>1350</v>
+        <v>1351</v>
       </c>
       <c r="C406" t="s">
-        <v>1351</v>
+        <v>1352</v>
       </c>
       <c r="D406" t="s">
         <v>69</v>
@@ -17838,13 +17841,13 @@
         <v>45</v>
       </c>
       <c r="G406" t="s">
-        <v>1352</v>
+        <v>1353</v>
       </c>
       <c r="H406" t="s">
         <v>38</v>
       </c>
       <c r="I406" t="s">
-        <v>1353</v>
+        <v>1354</v>
       </c>
       <c r="J406" t="s">
         <v>500</v>
@@ -17855,7 +17858,7 @@
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>1354</v>
+        <v>1355</v>
       </c>
       <c r="B407" t="s">
         <v>304</v>
@@ -17873,16 +17876,16 @@
         <v>45</v>
       </c>
       <c r="G407" t="s">
-        <v>1355</v>
+        <v>1356</v>
       </c>
       <c r="H407" t="s">
         <v>38</v>
       </c>
       <c r="I407" t="s">
-        <v>1331</v>
+        <v>1332</v>
       </c>
       <c r="J407" t="s">
-        <v>1331</v>
+        <v>1332</v>
       </c>
       <c r="K407" t="s">
         <v>2</v>
@@ -17893,10 +17896,10 @@
         <v>69701.0</v>
       </c>
       <c r="B408" t="s">
-        <v>1356</v>
+        <v>1357</v>
       </c>
       <c r="C408" t="s">
-        <v>1357</v>
+        <v>1358</v>
       </c>
       <c r="D408" t="s">
         <v>35</v>
@@ -17908,13 +17911,13 @@
         <v>52</v>
       </c>
       <c r="G408" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="H408" t="s">
         <v>47</v>
       </c>
       <c r="I408" t="s">
-        <v>1343</v>
+        <v>1344</v>
       </c>
       <c r="J408" t="s">
         <v>49</v>
@@ -17928,10 +17931,10 @@
         <v>67501.0</v>
       </c>
       <c r="B409" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
       <c r="C409" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="D409" t="s">
         <v>35</v>
@@ -17943,13 +17946,13 @@
         <v>45</v>
       </c>
       <c r="G409" t="s">
-        <v>1361</v>
+        <v>1362</v>
       </c>
       <c r="H409" t="s">
         <v>38</v>
       </c>
       <c r="I409" t="s">
-        <v>1353</v>
+        <v>1354</v>
       </c>
       <c r="J409" t="s">
         <v>500</v>
@@ -17963,10 +17966,10 @@
         <v>69301.0</v>
       </c>
       <c r="B410" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="C410" t="s">
-        <v>1363</v>
+        <v>1364</v>
       </c>
       <c r="D410" t="s">
         <v>35</v>
@@ -17978,13 +17981,13 @@
         <v>52</v>
       </c>
       <c r="G410" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="H410" t="s">
         <v>38</v>
       </c>
       <c r="I410" t="s">
-        <v>1353</v>
+        <v>1354</v>
       </c>
       <c r="J410" t="s">
         <v>500</v>
@@ -17998,10 +18001,10 @@
         <v>60001.0</v>
       </c>
       <c r="B411" t="s">
-        <v>1365</v>
+        <v>1366</v>
       </c>
       <c r="C411" t="s">
-        <v>1326</v>
+        <v>1327</v>
       </c>
       <c r="D411" t="s">
         <v>43</v>
@@ -18010,16 +18013,16 @@
         <v>43</v>
       </c>
       <c r="F411" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="G411" t="s">
-        <v>1327</v>
+        <v>1328</v>
       </c>
       <c r="H411" t="s">
         <v>47</v>
       </c>
       <c r="I411" t="s">
-        <v>1225</v>
+        <v>1226</v>
       </c>
       <c r="J411" t="s">
         <v>49</v>
@@ -18033,7 +18036,7 @@
         <v>74301.0</v>
       </c>
       <c r="B412" t="s">
-        <v>1366</v>
+        <v>1367</v>
       </c>
       <c r="C412" t="s">
         <v>310</v>
@@ -18048,16 +18051,16 @@
         <v>45</v>
       </c>
       <c r="G412" t="s">
-        <v>1367</v>
+        <v>1368</v>
       </c>
       <c r="H412" t="s">
         <v>38</v>
       </c>
       <c r="I412" t="s">
-        <v>1248</v>
+        <v>1249</v>
       </c>
       <c r="J412" t="s">
-        <v>1368</v>
+        <v>1369</v>
       </c>
       <c r="K412" t="s">
         <v>2</v>
@@ -18068,7 +18071,7 @@
         <v>74701.0</v>
       </c>
       <c r="B413" t="s">
-        <v>1369</v>
+        <v>1370</v>
       </c>
       <c r="C413" t="s">
         <v>804</v>
@@ -18083,16 +18086,16 @@
         <v>45</v>
       </c>
       <c r="G413" t="s">
-        <v>1370</v>
+        <v>1371</v>
       </c>
       <c r="H413" t="s">
         <v>38</v>
       </c>
       <c r="I413" t="s">
-        <v>1371</v>
+        <v>1372</v>
       </c>
       <c r="J413" t="s">
-        <v>1372</v>
+        <v>1373</v>
       </c>
       <c r="K413" t="s">
         <v>2</v>
@@ -18103,10 +18106,10 @@
         <v>72701.0</v>
       </c>
       <c r="B414" t="s">
-        <v>1373</v>
+        <v>1374</v>
       </c>
       <c r="C414" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="D414" t="s">
         <v>43</v>
@@ -18118,13 +18121,13 @@
         <v>139</v>
       </c>
       <c r="G414" t="s">
-        <v>1375</v>
+        <v>1376</v>
       </c>
       <c r="H414" t="s">
         <v>47</v>
       </c>
       <c r="I414" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
       <c r="J414" t="s">
         <v>49</v>
@@ -18138,7 +18141,7 @@
         <v>75901.0</v>
       </c>
       <c r="B415" t="s">
-        <v>1376</v>
+        <v>1377</v>
       </c>
       <c r="C415" t="s">
         <v>330</v>
@@ -18153,13 +18156,13 @@
         <v>45</v>
       </c>
       <c r="G415" t="s">
-        <v>1377</v>
+        <v>1378</v>
       </c>
       <c r="H415" t="s">
         <v>38</v>
       </c>
       <c r="I415" t="s">
-        <v>1378</v>
+        <v>1379</v>
       </c>
       <c r="J415" t="s">
         <v>740</v>
@@ -18173,10 +18176,10 @@
         <v>73901.0</v>
       </c>
       <c r="B416" t="s">
-        <v>1379</v>
+        <v>1380</v>
       </c>
       <c r="C416" t="s">
-        <v>1380</v>
+        <v>1381</v>
       </c>
       <c r="D416" t="s">
         <v>35</v>
@@ -18194,7 +18197,7 @@
         <v>38</v>
       </c>
       <c r="I416" t="s">
-        <v>1378</v>
+        <v>1379</v>
       </c>
       <c r="J416" t="s">
         <v>883</v>
@@ -18208,7 +18211,7 @@
         <v>71901.0</v>
       </c>
       <c r="B417" t="s">
-        <v>1381</v>
+        <v>1382</v>
       </c>
       <c r="C417" t="s">
         <v>813</v>
@@ -18223,16 +18226,16 @@
         <v>45</v>
       </c>
       <c r="G417" t="s">
-        <v>1382</v>
+        <v>1383</v>
       </c>
       <c r="H417" t="s">
         <v>38</v>
       </c>
       <c r="I417" t="s">
-        <v>1383</v>
+        <v>1384</v>
       </c>
       <c r="J417" t="s">
-        <v>1030</v>
+        <v>1031</v>
       </c>
       <c r="K417" t="s">
         <v>2</v>
@@ -18243,10 +18246,10 @@
         <v>73201.0</v>
       </c>
       <c r="B418" t="s">
-        <v>1276</v>
+        <v>1277</v>
       </c>
       <c r="C418" t="s">
-        <v>1277</v>
+        <v>1278</v>
       </c>
       <c r="D418" t="s">
         <v>35</v>
@@ -18264,7 +18267,7 @@
         <v>38</v>
       </c>
       <c r="I418" t="s">
-        <v>1384</v>
+        <v>1385</v>
       </c>
       <c r="J418" t="s">
         <v>718</v>
@@ -18278,10 +18281,10 @@
         <v>72501.0</v>
       </c>
       <c r="B419" t="s">
-        <v>1385</v>
+        <v>1386</v>
       </c>
       <c r="C419" t="s">
-        <v>1274</v>
+        <v>1275</v>
       </c>
       <c r="D419" t="s">
         <v>69</v>
@@ -18293,16 +18296,16 @@
         <v>52</v>
       </c>
       <c r="G419" t="s">
-        <v>1386</v>
+        <v>1387</v>
       </c>
       <c r="H419" t="s">
         <v>38</v>
       </c>
       <c r="I419" t="s">
-        <v>1387</v>
+        <v>1388</v>
       </c>
       <c r="J419" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="K419" t="s">
         <v>2</v>
@@ -18313,10 +18316,10 @@
         <v>74201.0</v>
       </c>
       <c r="B420" t="s">
-        <v>1388</v>
+        <v>1389</v>
       </c>
       <c r="C420" t="s">
-        <v>1389</v>
+        <v>1390</v>
       </c>
       <c r="D420" t="s">
         <v>43</v>
@@ -18328,13 +18331,13 @@
         <v>45</v>
       </c>
       <c r="G420" t="s">
-        <v>1390</v>
+        <v>1391</v>
       </c>
       <c r="H420" t="s">
         <v>38</v>
       </c>
       <c r="I420" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
       <c r="J420" t="s">
         <v>693</v>
@@ -18348,10 +18351,10 @@
         <v>71801.0</v>
       </c>
       <c r="B421" t="s">
-        <v>1391</v>
+        <v>1392</v>
       </c>
       <c r="C421" t="s">
-        <v>1392</v>
+        <v>1393</v>
       </c>
       <c r="D421" t="s">
         <v>43</v>
@@ -18363,13 +18366,13 @@
         <v>45</v>
       </c>
       <c r="G421" t="s">
-        <v>1393</v>
+        <v>1394</v>
       </c>
       <c r="H421" t="s">
         <v>38</v>
       </c>
       <c r="I421" t="s">
-        <v>1184</v>
+        <v>1185</v>
       </c>
       <c r="J421" t="s">
         <v>710</v>
@@ -18383,10 +18386,10 @@
         <v>73301.0</v>
       </c>
       <c r="B422" t="s">
-        <v>1394</v>
+        <v>1395</v>
       </c>
       <c r="C422" t="s">
-        <v>1395</v>
+        <v>1396</v>
       </c>
       <c r="D422" t="s">
         <v>43</v>
@@ -18398,13 +18401,13 @@
         <v>139</v>
       </c>
       <c r="G422" t="s">
-        <v>1396</v>
+        <v>1397</v>
       </c>
       <c r="H422" t="s">
         <v>47</v>
       </c>
       <c r="I422" t="s">
-        <v>1384</v>
+        <v>1385</v>
       </c>
       <c r="J422" t="s">
         <v>49</v>
@@ -18418,10 +18421,10 @@
         <v>73501.0</v>
       </c>
       <c r="B423" t="s">
-        <v>1397</v>
+        <v>1398</v>
       </c>
       <c r="C423" t="s">
-        <v>1398</v>
+        <v>1399</v>
       </c>
       <c r="D423" t="s">
         <v>43</v>
@@ -18433,13 +18436,13 @@
         <v>45</v>
       </c>
       <c r="G423" t="s">
-        <v>1399</v>
+        <v>1400</v>
       </c>
       <c r="H423" t="s">
         <v>38</v>
       </c>
       <c r="I423" t="s">
-        <v>1400</v>
+        <v>1401</v>
       </c>
       <c r="J423" t="s">
         <v>710</v>
@@ -18450,18 +18453,18 @@
     </row>
     <row r="426">
       <c r="A426" s="2" t="s">
-        <v>1401</v>
+        <v>1402</v>
       </c>
       <c r="B426" s="3" t="s">
-        <v>1402</v>
+        <v>1403</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="2" t="s">
-        <v>1403</v>
+        <v>1404</v>
       </c>
       <c r="B427" s="3" t="s">
-        <v>1404</v>
+        <v>1405</v>
       </c>
     </row>
   </sheetData>

</xml_diff>